<commit_message>
Update Google Forms links
</commit_message>
<xml_diff>
--- a/Психологический_центр_готово/01_Лабораторная_1_Сетевое_анкетирование/Лабораторная1_Ответы_анкеты.xlsx
+++ b/Психологический_центр_готово/01_Лабораторная_1_Сетевое_анкетирование/Лабораторная1_Ответы_анкеты.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ключ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ссылка" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ключ" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,6 +442,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Адрес Google Forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/forms/d/e/1FAIpQLScvyQ4Vzx3cxv3eQUqYjEYiqod6y7ALnRlsZYiTavVku9sEsA/viewform</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:BN4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1830,7 +1862,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add real Google Forms responses
</commit_message>
<xml_diff>
--- a/Психологический_центр_готово/01_Лабораторная_1_Сетевое_анкетирование/Лабораторная1_Ответы_анкеты.xlsx
+++ b/Психологический_центр_готово/01_Лабораторная_1_Сетевое_анкетирование/Лабораторная1_Ответы_анкеты.xlsx
@@ -8,8 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ссылка" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ключ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы Google Forms" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Обработка" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ключ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="m/d/yyyy h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -28,17 +33,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
+      <color theme="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -50,11 +56,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEDEA"/>
+        <fgColor rgb="00DCEAF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -62,20 +68,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
+    <border>
+      <left style="thin">
+        <color rgb="008A8F98"/>
+      </left>
+      <right style="thin">
+        <color rgb="008A8F98"/>
+      </right>
+      <top style="thin">
+        <color rgb="008A8F98"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="008A8F98"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -445,18 +475,18 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Адрес Google Forms</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>https://docs.google.com/forms/d/e/1FAIpQLScvyQ4Vzx3cxv3eQUqYjEYiqod6y7ALnRlsZYiTavVku9sEsA/viewform</t>
         </is>
@@ -473,424 +503,391 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN4"/>
+  <dimension ref="A1:BI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="8" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="8" customWidth="1" min="21" max="21"/>
-    <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="8" customWidth="1" min="23" max="23"/>
-    <col width="8" customWidth="1" min="24" max="24"/>
-    <col width="8" customWidth="1" min="25" max="25"/>
-    <col width="8" customWidth="1" min="26" max="26"/>
-    <col width="8" customWidth="1" min="27" max="27"/>
-    <col width="8" customWidth="1" min="28" max="28"/>
-    <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="8" customWidth="1" min="30" max="30"/>
-    <col width="8" customWidth="1" min="31" max="31"/>
-    <col width="8" customWidth="1" min="32" max="32"/>
-    <col width="8" customWidth="1" min="33" max="33"/>
-    <col width="8" customWidth="1" min="34" max="34"/>
-    <col width="8" customWidth="1" min="35" max="35"/>
-    <col width="8" customWidth="1" min="36" max="36"/>
-    <col width="8" customWidth="1" min="37" max="37"/>
-    <col width="8" customWidth="1" min="38" max="38"/>
-    <col width="8" customWidth="1" min="39" max="39"/>
-    <col width="8" customWidth="1" min="40" max="40"/>
-    <col width="8" customWidth="1" min="41" max="41"/>
-    <col width="8" customWidth="1" min="42" max="42"/>
-    <col width="8" customWidth="1" min="43" max="43"/>
-    <col width="8" customWidth="1" min="44" max="44"/>
-    <col width="8" customWidth="1" min="45" max="45"/>
-    <col width="8" customWidth="1" min="46" max="46"/>
-    <col width="8" customWidth="1" min="47" max="47"/>
-    <col width="8" customWidth="1" min="48" max="48"/>
-    <col width="8" customWidth="1" min="49" max="49"/>
-    <col width="8" customWidth="1" min="50" max="50"/>
-    <col width="8" customWidth="1" min="51" max="51"/>
-    <col width="8" customWidth="1" min="52" max="52"/>
-    <col width="8" customWidth="1" min="53" max="53"/>
-    <col width="8" customWidth="1" min="54" max="54"/>
-    <col width="8" customWidth="1" min="55" max="55"/>
-    <col width="8" customWidth="1" min="56" max="56"/>
-    <col width="8" customWidth="1" min="57" max="57"/>
-    <col width="8" customWidth="1" min="58" max="58"/>
-    <col width="8" customWidth="1" min="59" max="59"/>
-    <col width="8" customWidth="1" min="60" max="60"/>
-    <col width="8" customWidth="1" min="61" max="61"/>
-    <col width="8" customWidth="1" min="62" max="62"/>
-    <col width="8" customWidth="1" min="63" max="63"/>
-    <col width="8" customWidth="1" min="64" max="64"/>
-    <col width="8" customWidth="1" min="65" max="65"/>
-    <col width="8" customWidth="1" min="66" max="66"/>
-    <col width="16" customWidth="1" min="73" max="73"/>
-    <col width="10" customWidth="1" min="74" max="74"/>
-    <col width="46" customWidth="1" min="75" max="75"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="42" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="22" max="22"/>
+    <col width="42" customWidth="1" min="23" max="23"/>
+    <col width="39" customWidth="1" min="24" max="24"/>
+    <col width="38" customWidth="1" min="25" max="25"/>
+    <col width="42" customWidth="1" min="26" max="26"/>
+    <col width="42" customWidth="1" min="27" max="27"/>
+    <col width="42" customWidth="1" min="28" max="28"/>
+    <col width="42" customWidth="1" min="29" max="29"/>
+    <col width="42" customWidth="1" min="30" max="30"/>
+    <col width="42" customWidth="1" min="31" max="31"/>
+    <col width="40" customWidth="1" min="32" max="32"/>
+    <col width="42" customWidth="1" min="33" max="33"/>
+    <col width="42" customWidth="1" min="34" max="34"/>
+    <col width="42" customWidth="1" min="35" max="35"/>
+    <col width="39" customWidth="1" min="36" max="36"/>
+    <col width="42" customWidth="1" min="37" max="37"/>
+    <col width="42" customWidth="1" min="38" max="38"/>
+    <col width="42" customWidth="1" min="39" max="39"/>
+    <col width="42" customWidth="1" min="40" max="40"/>
+    <col width="42" customWidth="1" min="41" max="41"/>
+    <col width="36" customWidth="1" min="42" max="42"/>
+    <col width="42" customWidth="1" min="43" max="43"/>
+    <col width="39" customWidth="1" min="44" max="44"/>
+    <col width="42" customWidth="1" min="45" max="45"/>
+    <col width="39" customWidth="1" min="46" max="46"/>
+    <col width="42" customWidth="1" min="47" max="47"/>
+    <col width="42" customWidth="1" min="48" max="48"/>
+    <col width="42" customWidth="1" min="49" max="49"/>
+    <col width="40" customWidth="1" min="50" max="50"/>
+    <col width="42" customWidth="1" min="51" max="51"/>
+    <col width="42" customWidth="1" min="52" max="52"/>
+    <col width="37" customWidth="1" min="53" max="53"/>
+    <col width="42" customWidth="1" min="54" max="54"/>
+    <col width="42" customWidth="1" min="55" max="55"/>
+    <col width="42" customWidth="1" min="56" max="56"/>
+    <col width="28" customWidth="1" min="57" max="57"/>
+    <col width="39" customWidth="1" min="58" max="58"/>
+    <col width="42" customWidth="1" min="59" max="59"/>
+    <col width="42" customWidth="1" min="60" max="60"/>
+    <col width="42" customWidth="1" min="61" max="61"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Респондент</t>
+          <t>Отметка времени</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Возраст</t>
+          <t>1. Я могу долго работать без устали.</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Пол</t>
+          <t>2. Я всегда выполняю то, что обещаю, независимо от испытываемых в связи с этим неудобств.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>3. Как правило, руки и ноги у меня теплые.</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>4. Я редко страдаю от головных болей.</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>5. Я уверен в своих силах.</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>6. Ожидание раздражает меня.</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>7. Иногда я сам себе кажусь ни на что не годным.</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>8. В большинстве случаев я чувствую себя вполне счастливым.</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Q7</t>
+          <t>9. Мне трудно сосредоточиться на каком-то одном предмете.</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Q8</t>
+          <t>10. В детстве я с готовностью выполнял все данные мне поручения.</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>11. Не реже одного раза в месяц я страдаю от расстройства желудка.</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Q10</t>
+          <t>12. Я часто испытываю тревогу по какому-нибудь поводу.</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>13. Я не считаю себя более нервным, чем большинство людей.</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>14. Я не застенчив.</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>15. Жизнь для меня почти всегда связана с большим напряжением.</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>16. Иногда бывает, что я говорю о вещах, в которых не разбираюсь.</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>17. Я краснею не чаще, чем другие.</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>18. Я часто расстраиваюсь из-за пустяков.</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>19. Я редко замечаю у себя сердцебиение и одышку.</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Q18</t>
+          <t>20. Не все люди, которых я знаю, мне нравятся.</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>21. Я не могу уснуть, если меня что-то тревожит.</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Q20</t>
+          <t>22. Обычно я спокоен, и меня нелегко расстроить.</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Q21</t>
+          <t>23. Меня часто мучают ночные кошмары.</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Q22</t>
+          <t>24. Я склонен все принимать всерьез.</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Q23</t>
+          <t>25. Когда я нервничаю, у меня усиливается потливость.</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Q24</t>
+          <t>26. У меня беспокойный и прерывистый сон.</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Q25</t>
+          <t>27. В играх я предпочитаю скорее выигрывать, чем проигрывать.</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Q26</t>
+          <t>28. Я более чувствителен, чем большинство других людей.</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Q27</t>
+          <t>29. Бывает, что нескромные шутки и остроты вызывают у меня смех.</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Q28</t>
+          <t>30. Я хотел бы быть так же доволен жизнью, как, вероятно, довольны другие.</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Q29</t>
+          <t>31. Мой желудок сильно беспокоит меня.</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Q30</t>
+          <t>32. Я постоянно озабочен своими материальными и служебными делами.</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>Q31</t>
+          <t>33. Я настороженно отношусь к некоторым людям, хотя знаю, что они не могут причинить мне вреда.</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>Q32</t>
+          <t>34. Мне порой кажется, что передо мной нагромождены такие трудности, которых мне не преодолеть.</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>Q33</t>
+          <t>35. Я легко прихожу в замешательство.</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>Q34</t>
+          <t>36. Временами я становлюсь настолько возбужденным, что это мешает мне заснуть.</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>Q35</t>
+          <t>37. Я предпочитаю уклоняться от конфликтов и затруднительных положений.</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>Q36</t>
+          <t>38. У меня бывают приступы тошноты и рвоты.</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>Q37</t>
+          <t>39. Я никогда не опаздываю на свидания или работу.</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>Q38</t>
+          <t>40. Временами я определенно чувствую себя ненужным.</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>Q39</t>
+          <t>41. Иногда мне хочется выругаться.</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>Q40</t>
+          <t>42. Почти всегда я испытываю тревогу в связи с чем-либо или с кем-либо.</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>Q41</t>
+          <t>43. Меня беспокоят возможные неудачи.</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
         <is>
-          <t>Q42</t>
+          <t>44. Я часто боюсь, что вот-вот покраснею.</t>
         </is>
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>Q43</t>
+          <t>45. Меня нередко охватывает отчаяние.</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>Q44</t>
+          <t>46. Я — человек нервный и легко возбудимый.</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>Q45</t>
+          <t>47. Я часто замечаю, что мои руки дрожат, когда я пытаюсь что-нибудь сделать.</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
         <is>
-          <t>Q46</t>
+          <t>48. Я почти всегда испытываю чувство голода.</t>
         </is>
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>Q47</t>
+          <t>49. Мне не хватает уверенности в себе.</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
         <is>
-          <t>Q48</t>
+          <t>50. Я легко потею даже в прохладные дни.</t>
         </is>
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>Q49</t>
+          <t>51. Я часто мечтаю о таких вещах, о которых лучше никому не рассказывать.</t>
         </is>
       </c>
       <c r="BA1" s="1" t="inlineStr">
         <is>
-          <t>Q50</t>
+          <t>52. У меня очень редко болит живот.</t>
         </is>
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>Q51</t>
+          <t>53. Я считаю, что мне очень трудно сосредоточиться на какой-либо задаче или работе.</t>
         </is>
       </c>
       <c r="BC1" s="1" t="inlineStr">
         <is>
-          <t>Q52</t>
+          <t>54. У меня бывают периоды такого сильного беспокойства, что я не могу долго усидеть на одном месте.</t>
         </is>
       </c>
       <c r="BD1" s="1" t="inlineStr">
         <is>
-          <t>Q53</t>
+          <t>55. Я всегда отвечаю на письма сразу же после прочтения.</t>
         </is>
       </c>
       <c r="BE1" s="1" t="inlineStr">
         <is>
-          <t>Q54</t>
+          <t>56. Я легко расстраиваюсь.</t>
         </is>
       </c>
       <c r="BF1" s="1" t="inlineStr">
         <is>
-          <t>Q55</t>
+          <t>57. Я практически никогда не краснею.</t>
         </is>
       </c>
       <c r="BG1" s="1" t="inlineStr">
         <is>
-          <t>Q56</t>
+          <t>58. У меня гораздо меньше различных опасений и страхов, чем у моих друзей и знакомых.</t>
         </is>
       </c>
       <c r="BH1" s="1" t="inlineStr">
         <is>
-          <t>Q57</t>
+          <t>59. Бывает, что я откладываю на завтра то, что следует сделать сегодня.</t>
         </is>
       </c>
       <c r="BI1" s="1" t="inlineStr">
         <is>
-          <t>Q58</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>Q59</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>Q60</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>Баллы</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>Ложь</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>Интерпретация</t>
+          <t>60. Обычно я работаю с большим напряжением.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Респондент 1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>19</v>
+      <c r="A2" s="5" t="n">
+        <v>46149.0383775</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>женский</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -910,12 +907,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -925,12 +922,12 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -940,12 +937,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -955,22 +952,22 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
@@ -995,22 +992,22 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
@@ -1025,7 +1022,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -1050,12 +1047,12 @@
       </c>
       <c r="AI2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AK2" s="2" t="inlineStr">
@@ -1065,17 +1062,17 @@
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AO2" s="2" t="inlineStr">
@@ -1085,22 +1082,22 @@
       </c>
       <c r="AP2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AQ2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AR2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AS2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AT2" s="2" t="inlineStr">
@@ -1110,27 +1107,27 @@
       </c>
       <c r="AU2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AV2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AW2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AX2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AY2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AZ2" s="2" t="inlineStr">
@@ -1155,7 +1152,7 @@
       </c>
       <c r="BD2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="BE2" s="2" t="inlineStr">
@@ -1165,7 +1162,7 @@
       </c>
       <c r="BF2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BG2" s="2" t="inlineStr">
@@ -1175,48 +1172,27 @@
       </c>
       <c r="BH2" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BI2" s="2" t="inlineStr">
         <is>
           <t>Нет</t>
-        </is>
-      </c>
-      <c r="BJ2" s="2" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="BK2" s="2" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="BL2" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="BM2" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="BN2" s="2" t="inlineStr">
-        <is>
-          <t>очень высокий уровень тревоги; результаты могут быть недостоверными</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Респондент 2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>22</v>
+      <c r="A3" s="5" t="n">
+        <v>46149.10529356481</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>мужской</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1226,12 +1202,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1241,22 +1217,22 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -1266,17 +1242,17 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -1286,12 +1262,12 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -1311,7 +1287,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
@@ -1336,7 +1312,7 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr">
@@ -1361,7 +1337,7 @@
       </c>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AG3" s="2" t="inlineStr">
@@ -1376,7 +1352,7 @@
       </c>
       <c r="AI3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AJ3" s="2" t="inlineStr">
@@ -1386,7 +1362,7 @@
       </c>
       <c r="AK3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AL3" s="2" t="inlineStr">
@@ -1411,17 +1387,17 @@
       </c>
       <c r="AP3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AQ3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AR3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AS3" s="2" t="inlineStr">
@@ -1431,12 +1407,12 @@
       </c>
       <c r="AT3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AU3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AV3" s="2" t="inlineStr">
@@ -1451,22 +1427,22 @@
       </c>
       <c r="AX3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AY3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AZ3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BA3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BB3" s="2" t="inlineStr">
@@ -1486,7 +1462,7 @@
       </c>
       <c r="BE3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="BF3" s="2" t="inlineStr">
@@ -1506,53 +1482,32 @@
       </c>
       <c r="BI3" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="BJ3" s="2" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="BK3" s="2" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="BL3" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="BM3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="BN3" s="2" t="inlineStr">
-        <is>
-          <t>высокий уровень тревоги</t>
+          <t>Да</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Респондент 3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>20</v>
+      <c r="A4" s="5" t="n">
+        <v>46149.11082700232</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>женский</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1562,7 +1517,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1587,12 +1542,12 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1602,17 +1557,17 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -1622,22 +1577,22 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -1647,7 +1602,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -1667,12 +1622,12 @@
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AD4" s="2" t="inlineStr">
@@ -1687,7 +1642,7 @@
       </c>
       <c r="AF4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AG4" s="2" t="inlineStr">
@@ -1702,22 +1657,22 @@
       </c>
       <c r="AI4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AK4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
@@ -1732,17 +1687,17 @@
       </c>
       <c r="AO4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AP4" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="AQ4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AR4" s="2" t="inlineStr">
@@ -1757,7 +1712,7 @@
       </c>
       <c r="AT4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AU4" s="2" t="inlineStr">
@@ -1767,7 +1722,7 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="AW4" s="2" t="inlineStr">
@@ -1792,27 +1747,27 @@
       </c>
       <c r="BA4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BB4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BC4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BD4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BE4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BF4" s="2" t="inlineStr">
@@ -1822,7 +1777,7 @@
       </c>
       <c r="BG4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="BH4" s="2" t="inlineStr">
@@ -1833,27 +1788,6 @@
       <c r="BI4" s="2" t="inlineStr">
         <is>
           <t>Да</t>
-        </is>
-      </c>
-      <c r="BJ4" s="2" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="BK4" s="2" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="BL4" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="BM4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="BN4" s="2" t="inlineStr">
-        <is>
-          <t>средний уровень тревоги с тенденцией к низкому; результаты могут быть недостоверными</t>
         </is>
       </c>
     </row>
@@ -1868,113 +1802,1612 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:BM4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="39" max="39"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
+    <col width="12" customWidth="1" min="51" max="51"/>
+    <col width="12" customWidth="1" min="52" max="52"/>
+    <col width="12" customWidth="1" min="53" max="53"/>
+    <col width="12" customWidth="1" min="54" max="54"/>
+    <col width="12" customWidth="1" min="55" max="55"/>
+    <col width="12" customWidth="1" min="56" max="56"/>
+    <col width="12" customWidth="1" min="57" max="57"/>
+    <col width="12" customWidth="1" min="58" max="58"/>
+    <col width="12" customWidth="1" min="59" max="59"/>
+    <col width="12" customWidth="1" min="60" max="60"/>
+    <col width="12" customWidth="1" min="61" max="61"/>
+    <col width="12" customWidth="1" min="62" max="62"/>
+    <col width="12" customWidth="1" min="63" max="63"/>
+    <col width="12" customWidth="1" min="64" max="64"/>
+    <col width="42" customWidth="1" min="65" max="65"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Респондент</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Отметка времени</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Q20</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Q21</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Q22</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Q23</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Q24</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Q25</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Q26</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Q27</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Q28</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Q29</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Q30</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Q31</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Q32</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Q33</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Q34</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Q35</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Q36</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Q37</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Q38</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Q39</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Q40</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Q41</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Q42</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Q43</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Q44</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Q45</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>Q46</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Q47</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Q48</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Q49</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Q50</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Q51</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>Q52</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Q53</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Q54</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Q55</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Q56</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Q57</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Q58</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>Q59</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>Q60</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>Баллы</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Ложь</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Интерпретация</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Респондент 1</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46149.0383775</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AO2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AR2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AS2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AT2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AW2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AX2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AY2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AZ2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BA2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BB2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BC2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BD2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BE2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BF2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BG2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BH2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BI2" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BJ2" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BK2" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="BL2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM2" s="2" t="inlineStr">
+        <is>
+          <t>средний уровень тревоги с тенденцией к высокому</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Респондент 2</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>46149.10529356481</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AI3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AK3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AO3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AP3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AQ3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AR3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AS3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AT3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AU3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AV3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AW3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AX3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AY3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AZ3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BA3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BB3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BC3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BD3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BE3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BF3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BG3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BH3" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BI3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BJ3" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BK3" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="BL3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="BM3" s="2" t="inlineStr">
+        <is>
+          <t>высокий уровень тревоги</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Респондент 3</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>46149.11082700232</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AG4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AI4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AK4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AL4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AM4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AN4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AO4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AP4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AQ4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AR4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AS4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AT4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AU4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AV4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AW4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AX4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AY4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AZ4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BA4" s="2" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="BB4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BC4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BD4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BE4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BF4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BG4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BH4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BI4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BJ4" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="BK4" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="BL4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="BM4" s="2" t="inlineStr">
+        <is>
+          <t>высокий уровень тревоги; результаты могут быть недостоверными</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Номера вопросов</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Правило</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Баллы за ответ Да</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>6, 7, 9, 11, 12, 13, 15, 18, 21, 23, 24, 25, 26, 28, 30, 31, 32, 33, 34, 35, 36, 37, 38, 40, 42, 44, 45, 46, 47, 48, 49, 50, 53, 54, 56, 60</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>+1 балл</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Баллы за ответ Нет</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>1, 3, 4, 5, 8, 14, 17, 19, 22, 39, 43, 52, 57, 58</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>+1 балл</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Контроль ложь Да</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2, 10, 55</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>считать как показатель недостоверности</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Контроль ложь Нет</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>16, 20, 27, 29, 41, 51, 59</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>считать как показатель недостоверности</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Интерпретация</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>0-5; 5-15; 15-25; 25-40; 40-50</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>низкий; средний-низкий; средний-высокий; высокий; очень высокий</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Количество реальных ответов</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Период ответов</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>07.05.2026 00:55 - 07.05.2026 02:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Средний балл тревожности</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Минимальный балл</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Максимальный балл</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Средний показатель контроля</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Респондент 1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>18 баллов; контроль 2; средний уровень тревоги с тенденцией к высокому</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Респондент 2</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>31 балл; контроль 4; высокий уровень тревоги</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Респондент 3</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>29 баллов; контроль 6; высокий уровень тревоги; результаты могут быть недостоверными</t>
         </is>
       </c>
     </row>

</xml_diff>